<commit_message>
All files are cleaned except "feature_adder.py"
</commit_message>
<xml_diff>
--- a/src/models/prediction/one_day_input.xlsx
+++ b/src/models/prediction/one_day_input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\ML_project\bargh\src\models\prediction\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\ML_project\Bargh_ML\src\models\prediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519D9B09-1820-43BC-A0A1-EB39BECAB66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DD162C-173E-4BA0-B217-7EF598E02223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{49E3F3CD-7BB1-4BC2-A851-C7129C1E0EE9}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="8">
   <si>
     <t>name</t>
   </si>
@@ -34,31 +34,16 @@
     <t>hour</t>
   </si>
   <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>forecast</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
     <t>پرند</t>
   </si>
   <si>
-    <t>L</t>
+    <t>G11</t>
   </si>
   <si>
-    <t>SO</t>
+    <t>temp_sens</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>G11</t>
+    <t>G12</t>
   </si>
 </sst>
 </file>
@@ -918,13 +903,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0ABECAF-C87E-4F60-BC79-F90905C7BF97}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -938,569 +924,827 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D11">
+        <v>10</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D13">
         <v>12</v>
       </c>
-      <c r="C2" s="1">
-        <v>45929</v>
-      </c>
-      <c r="D2">
+      <c r="E13">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D16">
+        <v>15</v>
+      </c>
+      <c r="E16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D17">
+        <v>16</v>
+      </c>
+      <c r="E17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D18">
+        <v>17</v>
+      </c>
+      <c r="E18">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D19">
+        <v>18</v>
+      </c>
+      <c r="E19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D20">
+        <v>19</v>
+      </c>
+      <c r="E20">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D21">
+        <v>20</v>
+      </c>
+      <c r="E21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D22">
+        <v>21</v>
+      </c>
+      <c r="E22">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D23">
+        <v>22</v>
+      </c>
+      <c r="E23">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D24">
+        <v>23</v>
+      </c>
+      <c r="E24">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>5</v>
+      </c>
+      <c r="C25" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D25">
         <v>24</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D30">
+        <v>5</v>
+      </c>
+      <c r="E30">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D31">
+        <v>6</v>
+      </c>
+      <c r="E31">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D32">
+        <v>7</v>
+      </c>
+      <c r="E32">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D33">
+        <v>8</v>
+      </c>
+      <c r="E33">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D34">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D35">
         <v>10</v>
       </c>
-      <c r="F2">
-        <v>30188</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="E35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D36">
+        <v>11</v>
+      </c>
+      <c r="E36">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D37">
         <v>12</v>
       </c>
-      <c r="C3" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3">
-        <v>29288</v>
-      </c>
-      <c r="G3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4">
-        <v>28138</v>
-      </c>
-      <c r="G4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5">
-        <v>27300</v>
-      </c>
-      <c r="G5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>26788</v>
-      </c>
-      <c r="G6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7">
-        <v>26500</v>
-      </c>
-      <c r="G7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D8">
-        <v>6</v>
-      </c>
-      <c r="E8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8">
-        <v>26298</v>
-      </c>
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D9">
-        <v>7</v>
-      </c>
-      <c r="E9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9">
-        <v>24876</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D10">
-        <v>8</v>
-      </c>
-      <c r="E10" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10">
-        <v>24871</v>
-      </c>
-      <c r="G10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D11">
-        <v>9</v>
-      </c>
-      <c r="E11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11">
-        <v>24892</v>
-      </c>
-      <c r="G11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D12">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12">
-        <v>25669</v>
-      </c>
-      <c r="G12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D13">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13">
-        <v>26414</v>
-      </c>
-      <c r="G13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D14">
-        <v>12</v>
-      </c>
-      <c r="E14" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14">
-        <v>26887</v>
-      </c>
-      <c r="G14" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D15">
+      <c r="E37">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D38">
         <v>13</v>
       </c>
-      <c r="E15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15">
-        <v>27049</v>
-      </c>
-      <c r="G15" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B16" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D16">
+      <c r="E38">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D39">
         <v>14</v>
       </c>
-      <c r="E16" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16">
-        <v>27087</v>
-      </c>
-      <c r="G16" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D17">
+      <c r="E39">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D40">
         <v>15</v>
       </c>
-      <c r="E17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17">
-        <v>26830</v>
-      </c>
-      <c r="G17" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D18">
+      <c r="E40">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D41">
         <v>16</v>
       </c>
-      <c r="E18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18">
-        <v>26586</v>
-      </c>
-      <c r="G18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D19">
+      <c r="E41">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D42">
         <v>17</v>
       </c>
-      <c r="E19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19">
-        <v>26796</v>
-      </c>
-      <c r="G19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D20">
+      <c r="E42">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D43">
         <v>18</v>
       </c>
-      <c r="E20" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20">
-        <v>27380</v>
-      </c>
-      <c r="G20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>7</v>
-      </c>
-      <c r="B21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D21">
+      <c r="E43">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>4</v>
+      </c>
+      <c r="B44" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D44">
         <v>19</v>
       </c>
-      <c r="E21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21">
-        <v>30182</v>
-      </c>
-      <c r="G21" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D22">
-        <v>20</v>
-      </c>
-      <c r="E22" t="s">
-        <v>10</v>
-      </c>
-      <c r="F22">
-        <v>31946</v>
-      </c>
-      <c r="G22" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" t="s">
-        <v>12</v>
-      </c>
-      <c r="C23" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D23">
+      <c r="E44">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D45">
+        <v>20</v>
+      </c>
+      <c r="E45">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D46">
         <v>21</v>
       </c>
-      <c r="E23" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23">
-        <v>32062</v>
-      </c>
-      <c r="G23" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D24">
+      <c r="E46">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>4</v>
+      </c>
+      <c r="B47" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D47">
         <v>22</v>
       </c>
-      <c r="E24" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24">
-        <v>31746</v>
-      </c>
-      <c r="G24" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="1">
-        <v>45930</v>
-      </c>
-      <c r="D25">
+      <c r="E47">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>4</v>
+      </c>
+      <c r="B48" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D48">
         <v>23</v>
       </c>
-      <c r="E25" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25">
-        <v>31236</v>
-      </c>
-      <c r="G25" t="s">
-        <v>9</v>
+      <c r="E48">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" s="1">
+        <v>45943</v>
+      </c>
+      <c r="D49">
+        <v>24</v>
+      </c>
+      <c r="E49">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G25">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D25">
     <sortCondition ref="B3:B25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Before changing the structures
</commit_message>
<xml_diff>
--- a/src/models/prediction/one_day_input.xlsx
+++ b/src/models/prediction/one_day_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\ML_project\Bargh_ML\src\models\prediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961B1B2C-9E8E-4F62-AA4A-070BF34633E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8442332-EF75-4FEC-91F2-3D488C9776FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{49E3F3CD-7BB1-4BC2-A851-C7129C1E0EE9}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="8">
   <si>
     <t>name</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>G12</t>
+  </si>
+  <si>
+    <t>قم</t>
   </si>
 </sst>
 </file>
@@ -922,7 +925,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>

</xml_diff>